<commit_message>
Add the lab tour and biosafety video; defer picking
lab_tour and biosafety are the two halves of the safety video from
reshoot/01-safety.md - a continuous walking shot and a static take at a
bench. Separate takes, one video, so two slates.

Picking is off tomorrow for want of time. bestp_pick and pp6_pick move to
a 'Later' section; the plates go into the fridge instead, which makes
parafilm the load-bearing item of the day rather than housekeeping. Its
slate now says why the plates are being sealed, and that a week is the
window before satellites and fading green start costing you.

Day 2 is now lab_tour, biosafety, ctrl_read, parafilm.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video_plans/shoot_protocols_plan.xlsx
+++ b/video_plans/shoot_protocols_plan.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.1640625" customWidth="1" min="1" max="1"/>
@@ -492,22 +492,22 @@
       </c>
     </row>
     <row r="2" customFormat="1" s="3">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>agar_fresh</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Preparation of LB Agar (250 mL bottles)</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>3 bottles, plus empty bottles</t>
         </is>
@@ -517,25 +517,24 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3" customFormat="1" s="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>broth_2yt</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Preparation of 2YT Broth (250 mL bottles)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>4 bottles</t>
         </is>
@@ -545,30 +544,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4" customFormat="1" s="3">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>abx_carb</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Preparation of Antibiotic 1000x Stock</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>100 mg/mL</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>mg x 10, water</t>
         </is>
@@ -578,30 +576,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5" customFormat="1" s="3">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>abx_spec</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Preparation of Antibiotic 1000x Stock</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>100 mg/mL</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>mg x 10, water</t>
         </is>
@@ -611,30 +608,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6" customFormat="1" s="3">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>abx_kan</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Preparation of Antibiotic 1000x Stock</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>25 mg/mL</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>mg x 40, water</t>
         </is>
@@ -644,30 +640,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7" customFormat="1" s="3">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>abx_erm</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Preparation of Antibiotic 1000x Stock</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>100 mg/mL</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>mg x 10, ethanol</t>
         </is>
@@ -677,25 +672,24 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8" customFormat="1" s="3">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>agar_remelt</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Re-melting Solidified LB Agar</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>1 bottle</t>
         </is>
@@ -705,25 +699,24 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9" customFormat="1" s="3">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>pour_many_plates</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Pouring many Carb petri dishes</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Carb, 1 stack</t>
         </is>
@@ -738,25 +731,24 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10" customFormat="1" s="3">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>pour_few_plates1</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Pouring a few Erm petri dishes with conicol</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Erm, 3 plates</t>
         </is>
@@ -771,25 +763,24 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11" customFormat="1" s="3">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>pour_few_plates2</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Pouring a few spec petri dishes with bottle</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>Spec, 4 plates</t>
         </is>
@@ -804,25 +795,23 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12" customFormat="1" s="3">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>pour_large_plate</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Pouring and Spreading Large Petri Dishes (150 mm)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>150 mm plates; existing module</t>
@@ -845,22 +834,22 @@
       </c>
     </row>
     <row r="13" customFormat="1" s="3">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>(no vid)</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Pouring a few kan petri dishes</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Kan, 3 plates</t>
         </is>
@@ -872,22 +861,22 @@
       </c>
     </row>
     <row r="14" customFormat="1" s="3">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>(no vid)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Pouring a few plain petri dishes</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>no ab, 3 plates</t>
         </is>
@@ -899,27 +888,27 @@
       </c>
     </row>
     <row r="15" customFormat="1" s="3">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>ctrl_streak</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Streaking control strain</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>vid 1: 3 plates do all 4</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>neg, streak, and put carb one on spec, streak and neg for others</t>
         </is>
@@ -941,27 +930,27 @@
       </c>
     </row>
     <row r="16" customFormat="1" s="3">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>ctrl_transform1</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Label plates, thaw cells, incubate dna</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>4 reactions</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>each control plasmid (carb, kan, spec, erm) — same for all four; the fork is at step 2</t>
         </is>
@@ -976,30 +965,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17" customFormat="1" s="2">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>ctrl_transform2a</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Heat shock and plate</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>1 reaction</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>carb only — no rescue, plate straight away</t>
         </is>
@@ -1014,30 +1002,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18" customFormat="1" s="2">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>ctrl_transform2b</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Heat shock and rescue</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>3 reactions</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>kan, spec, erm — 200 uL 2YT, 37 C, 1 h; do not plate yet</t>
         </is>
@@ -1052,30 +1039,29 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>ctrl_transform3a</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Plate from a rescue</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>controls</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>3 reactions</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>kan, spec, erm — plate all the liquid; dry before inverting</t>
         </is>
@@ -1097,22 +1083,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>bestP_transform1</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Label plates, thaw cells, incubate dna</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>7 reactions, on carb</t>
         </is>
@@ -1134,22 +1120,22 @@
       </c>
     </row>
     <row r="21" customFormat="1" s="3">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>bestP_transform2a</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Heat shock and plate</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>7 reactions, on carb</t>
         </is>
@@ -1184,90 +1170,115 @@
       </c>
     </row>
     <row r="24" customFormat="1" s="1">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>lab_tour</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lab tour</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>one continuous walking shot</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>room must be quiet; say every location out loud</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>safety video</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>biosafety</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lab rules and biosafety</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>static, at a bench</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>the six must-say lines map onto quiz questions</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>safety video</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>parafilm</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Sealing Petri Dishes with Parafilm</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="1" s="2">
+      <c r="A27" t="inlineStr">
         <is>
           <t>ctrl_read</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Examine and photograph plates</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>controls video</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>bestp_pick</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Pick bestP's colonies into a block</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>bestp</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Full block</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>BestP video</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" customFormat="1" s="2">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>pp6_pick</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Pick pp6 clones into a 15mL conicol</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>pp6</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>do 2</t>
         </is>
       </c>
     </row>
@@ -1275,29 +1286,29 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Day 3</t>
+          <t>Later — plates held in the fridge</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="2">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>bestp_tecan</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Tecan the bestp's from a block</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>bestp_pick</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Pick bestP's colonies into a block</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>56 wells</t>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Full block</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1306,31 +1317,87 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>pp6_pick</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pick pp6 clones into a 15mL conicol</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>pp6</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>do 2</t>
+        </is>
+      </c>
+    </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>bestp_tecan</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tecan the bestp's from a block</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>bestp</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>56 wells</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>BestP video</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Whenever</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>bestp_intro</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>BestP video</t>
         </is>
@@ -1347,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.1640625" customWidth="1" min="1" max="1"/>
@@ -1424,7 +1491,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3" customFormat="1" s="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1452,7 +1518,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4" customFormat="1" s="3">
       <c r="A4" s="3" t="inlineStr">
@@ -1485,7 +1550,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5" customFormat="1" s="3">
       <c r="A5" s="3" t="inlineStr">
@@ -1518,7 +1582,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6" customFormat="1" s="3">
       <c r="A6" s="3" t="inlineStr">
@@ -1551,7 +1614,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7" customFormat="1" s="3">
       <c r="A7" s="3" t="inlineStr">
@@ -1584,7 +1646,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8" customFormat="1" s="3">
       <c r="A8" s="3" t="inlineStr">
@@ -1612,7 +1673,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9" customFormat="1" s="3">
       <c r="A9" s="3" t="inlineStr">
@@ -1645,7 +1705,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10" customFormat="1" s="3">
       <c r="A10" s="3" t="inlineStr">
@@ -1678,7 +1737,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11" customFormat="1" s="3">
       <c r="A11" s="3" t="inlineStr">
@@ -1711,7 +1769,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12" customFormat="1" s="3">
       <c r="A12" s="4" t="inlineStr">
@@ -1883,7 +1940,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17" customFormat="1" s="3">
       <c r="A17" s="3" t="inlineStr">
@@ -1921,7 +1977,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18" customFormat="1" s="3">
       <c r="A18" s="4" t="inlineStr">
@@ -1959,7 +2014,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19" customFormat="1" s="2">
       <c r="A19" s="4" t="inlineStr">
@@ -2004,97 +2058,127 @@
       </c>
     </row>
     <row r="20" customFormat="1" s="2">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>lab_tour</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Lab tour</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>one continuous walking shot</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>room must be quiet; say every location out loud</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>safety video</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="1" s="2">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>biosafety</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Lab rules and biosafety</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>static, at a bench</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>the six must-say lines map onto quiz questions</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>safety video</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" customFormat="1" s="2">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>parafilm</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Sealing Petri Dishes with Parafilm</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" customFormat="1" s="2">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" customFormat="1" s="2">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>ctrl_read</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Examine and photograph plates</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>controls video</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" customFormat="1" s="2">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>bestp_intro</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>(none)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>bestp</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>BestP video</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" customFormat="1" s="2">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>(agar_fresh)</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Preparation of LB Agar (250 mL bottles)</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>bestp</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="24" customFormat="1" s="2">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>(pour_many_plates)</t>
+          <t>bestp_intro</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Pouring Standard Petri Dishes</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2111,12 +2195,12 @@
     <row r="25" customFormat="1" s="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>bestP_transform1</t>
+          <t>(agar_fresh)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Label plates, thaw cells, incubate dna</t>
+          <t>Preparation of LB Agar (250 mL bottles)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2124,36 +2208,21 @@
           <t>bestp</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>7 reactions, on carb</t>
-        </is>
-      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>covered by ctrl_transform1 — pJ01/pJ12/pJ19 were transformed there</t>
+          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="26" customFormat="1" s="2">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>bestP_transform2a</t>
+          <t>(pour_many_plates)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Heat shock and plate</t>
+          <t>Pouring Standard Petri Dishes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2161,41 +2230,21 @@
           <t>bestp</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>7 reactions, on carb</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>carb — no rescue</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>covered by ctrl_transform2a/2b; three references explain BestP without repeating the whole run</t>
+          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>bestp_pick</t>
+          <t>bestP_transform1</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Pick bestP's colonies into a block</t>
+          <t>Label plates, thaw cells, incubate dna</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2205,59 +2254,138 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Full block</t>
+          <t>7 reactions, on carb</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>BestP video</t>
+          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>covered by ctrl_transform1 — pJ01/pJ12/pJ19 were transformed there</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>pp6_pick</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="inlineStr">
-        <is>
-          <t>Pick pp6 clones into a 15mL conicol</t>
-        </is>
-      </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>pp6</t>
-        </is>
-      </c>
-      <c r="D28" s="1" t="inlineStr">
-        <is>
-          <t>do 2</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>bestP_transform2a</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Heat shock and plate</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>bestp</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>7 reactions, on carb</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>carb — no rescue</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>covered by ctrl_transform2a/2b; three references explain BestP without repeating the whole run</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>bestp_pick</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Pick bestP's colonies into a block</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>bestp</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Full block</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>BestP video</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>pp6_pick</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>Pick pp6 clones into a 15mL conicol</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>pp6</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>do 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>bestp_tecan</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Tecan the bestp's from a block</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>56 wells</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>BestP video</t>
         </is>

</xml_diff>

<commit_message>
Add ctrl_intro; name the fridge on the parafilm slate
Today is four clips: lab_tour, ctrl_intro, ctrl_read, parafilm.

ctrl_intro is new - what a control strain is and why the lab keeps them,
no bench work. It takes the conceptual opening that had been buried in
the ctrl_streak slate and gives it its own clip, which also sets up the
streak and transformation footage already shot.

parafilm now names the destination. storage.json distinguishes the
Culture Fridge, for active cultures and plates with cells on them, from
the Main / Cell-Free fridge, for sterile dishes, DMEM and gels. Saying
which and why is more use than saying 'the fridge'.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video_plans/shoot_protocols_plan.xlsx
+++ b/video_plans/shoot_protocols_plan.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.1640625" customWidth="1" min="1" max="1"/>
@@ -1209,158 +1209,201 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>parafilm</t>
+          <t>ctrl_intro</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sealing Petri Dishes with Parafilm</t>
+          <t>What control strains are and why we keep them</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>general</t>
-        </is>
-      </c>
+          <t>controls</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>no bench work</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>intro to the controls thread; sets up the streak and transformation clips</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>controls video</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>parafilm</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Sealing Petri Dishes with Parafilm</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>store in the Culture Fridge (4 °C), not the Main/Cell-Free fridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" customFormat="1" s="2">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>ctrl_read</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Examine and photograph plates</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>general</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>controls video</t>
         </is>
       </c>
     </row>
-    <row r="27" customFormat="1" s="2"/>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Day 3</t>
-        </is>
-      </c>
-    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>bestp_pick</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Pick bestP's colonies into a block</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>bestp</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Full block</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>BestP video</t>
+          <t>Day 3</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="1" s="2">
       <c r="A30" t="inlineStr">
         <is>
-          <t>pp6_pick</t>
+          <t>bestp_pick</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pick pp6 clones into a 15mL conicol</t>
+          <t>Pick bestP's colonies into a block</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pp6</t>
+          <t>bestp</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>do 2</t>
+          <t>Full block</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4</t>
+          <t>pp6_pick</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pick pp6 clones into a 15mL conicol</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>pp6</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>do 2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Day 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>bestp_tecan</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Tecan the bestp's from a block</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>56 wells</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>BestP video</t>
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Whenever</t>
-        </is>
-      </c>
-    </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Whenever</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>bestp_intro</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>BestP video</t>
         </is>
@@ -1377,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.1640625" customWidth="1" min="1" max="1"/>
@@ -2059,29 +2102,50 @@
     <row r="21" customFormat="1" s="2">
       <c r="A21" t="inlineStr">
         <is>
-          <t>parafilm</t>
+          <t>ctrl_intro</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sealing Petri Dishes with Parafilm</t>
+          <t>What control strains are and why we keep them</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>general</t>
-        </is>
-      </c>
+          <t>controls</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>no bench work</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>intro to the controls thread; sets up the streak and transformation clips</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>controls video</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22" customFormat="1" s="2">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ctrl_read</t>
+          <t>parafilm</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Examine and photograph plates</t>
+          <t>Sealing Petri Dishes with Parafilm</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2089,43 +2153,43 @@
           <t>general</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>controls video</t>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>store in the Culture Fridge (4 °C), not the Main/Cell-Free fridge</t>
         </is>
       </c>
     </row>
     <row r="23" customFormat="1" s="2">
       <c r="A23" t="inlineStr">
         <is>
-          <t>bestp_intro</t>
+          <t>ctrl_read</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>(none)</t>
+          <t>Examine and photograph plates</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>bestp</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>BestP video</t>
+          <t>controls video</t>
         </is>
       </c>
     </row>
     <row r="24" customFormat="1" s="2">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(agar_fresh)</t>
+          <t>bestp_intro</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Preparation of LB Agar (250 mL bottles)</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2142,12 +2206,12 @@
     <row r="25" customFormat="1" s="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(pour_many_plates)</t>
+          <t>(agar_fresh)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pouring Standard Petri Dishes</t>
+          <t>Preparation of LB Agar (250 mL bottles)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2164,12 +2228,12 @@
     <row r="26" customFormat="1" s="2">
       <c r="A26" t="inlineStr">
         <is>
-          <t>bestP_transform1</t>
+          <t>(pour_many_plates)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Label plates, thaw cells, incubate dna</t>
+          <t>Pouring Standard Petri Dishes</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2177,36 +2241,21 @@
           <t>bestp</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>7 reactions, on carb</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>covered by ctrl_transform1 — pJ01/pJ12/pJ19 were transformed there</t>
+          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>bestP_transform2a</t>
+          <t>bestP_transform1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Heat shock and plate</t>
+          <t>Label plates, thaw cells, incubate dna</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2219,11 +2268,6 @@
           <t>7 reactions, on carb</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>carb — no rescue</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>not filmed — BestP reuses the minipreps-into-cells video</t>
@@ -2236,19 +2280,19 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>covered by ctrl_transform2a/2b; three references explain BestP without repeating the whole run</t>
+          <t>covered by ctrl_transform1 — pJ01/pJ12/pJ19 were transformed there</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>bestp_pick</t>
+          <t>bestP_transform2a</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pick bestP's colonies into a block</t>
+          <t>Heat shock and plate</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2258,59 +2302,101 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Full block</t>
+          <t>7 reactions, on carb</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>carb — no rescue</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>BestP video</t>
+          <t>not filmed — BestP reuses the minipreps-into-cells video</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>covered by ctrl_transform2a/2b; three references explain BestP without repeating the whole run</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>pp6_pick</t>
+          <t>bestp_pick</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pick pp6 clones into a 15mL conicol</t>
+          <t>Pick bestP's colonies into a block</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pp6</t>
+          <t>bestp</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>do 2</t>
+          <t>Full block</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>BestP video</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>pp6_pick</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Pick pp6 clones into a 15mL conicol</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>pp6</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>do 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>bestp_tecan</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Tecan the bestp's from a block</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>bestp</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>56 wells</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>BestP video</t>
         </is>

</xml_diff>